<commit_message>
Today's drafts, rebuilt on the swept code
Nineteen company emails and every image-body report re-made so what is
on disk matches what the code now does: the shut curve inside the frame
with its date axis, the four figures under it, the position paragraphs
that count in singular and plural, the all-clear story in the body, and
alt text on every inline picture.

CHECK_REPORTS: PASS - 61 pages, 31 drafts, every body clean.
TEST_DAILY_PACKS 2026-08-05: 363 passed, 0 failed.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017cvkBVSy5jN5HGmHFYEnYK
</commit_message>
<xml_diff>
--- a/01_Reporting_Suite/K2 DAILY REPORTING/02 EMAIL CONTROL/Email Control Register.xlsx
+++ b/01_Reporting_Suite/K2 DAILY REPORTING/02 EMAIL CONTROL/Email Control Register.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M82"/>
+  <dimension ref="A1:M99"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3948,8 +3948,6 @@
           <t>thomas.maher@coates.com.au; cody.mitchell@coates.com.au; benjamin.vandenbroek@cemaust.com.au; david.moore@cemaust.com.au; John.Pickels@cemaust.com.au</t>
         </is>
       </c>
-      <c r="I65" t="inlineStr"/>
-      <c r="J65" t="inlineStr"/>
       <c r="K65" t="n">
         <v>0</v>
       </c>
@@ -4001,8 +3999,6 @@
           <t>thomas.maher@coates.com.au; cody.mitchell@coates.com.au; benjamin.vandenbroek@cemaust.com.au; david.moore@cemaust.com.au; John.Pickels@cemaust.com.au</t>
         </is>
       </c>
-      <c r="I66" t="inlineStr"/>
-      <c r="J66" t="inlineStr"/>
       <c r="K66" t="n">
         <v>0</v>
       </c>
@@ -4054,8 +4050,6 @@
           <t>thomas.maher@coates.com.au; cody.mitchell@coates.com.au; benjamin.vandenbroek@cemaust.com.au; david.moore@cemaust.com.au; John.Pickels@cemaust.com.au</t>
         </is>
       </c>
-      <c r="I67" t="inlineStr"/>
-      <c r="J67" t="inlineStr"/>
       <c r="K67" t="n">
         <v>0</v>
       </c>
@@ -4107,8 +4101,6 @@
           <t>thomas.maher@coates.com.au; cody.mitchell@coates.com.au; benjamin.vandenbroek@cemaust.com.au; david.moore@cemaust.com.au; John.Pickels@cemaust.com.au</t>
         </is>
       </c>
-      <c r="I68" t="inlineStr"/>
-      <c r="J68" t="inlineStr"/>
       <c r="K68" t="n">
         <v>0</v>
       </c>
@@ -4160,8 +4152,6 @@
           <t>thomas.maher@coates.com.au; cody.mitchell@coates.com.au; benjamin.vandenbroek@cemaust.com.au; david.moore@cemaust.com.au; John.Pickels@cemaust.com.au</t>
         </is>
       </c>
-      <c r="I69" t="inlineStr"/>
-      <c r="J69" t="inlineStr"/>
       <c r="K69" t="n">
         <v>0</v>
       </c>
@@ -4213,8 +4203,6 @@
           <t>thomas.maher@coates.com.au; cody.mitchell@coates.com.au; benjamin.vandenbroek@cemaust.com.au; david.moore@cemaust.com.au; John.Pickels@cemaust.com.au</t>
         </is>
       </c>
-      <c r="I70" t="inlineStr"/>
-      <c r="J70" t="inlineStr"/>
       <c r="K70" t="n">
         <v>0</v>
       </c>
@@ -4266,8 +4254,6 @@
           <t>thomas.maher@coates.com.au; cody.mitchell@coates.com.au; benjamin.vandenbroek@cemaust.com.au; david.moore@cemaust.com.au; John.Pickels@cemaust.com.au</t>
         </is>
       </c>
-      <c r="I71" t="inlineStr"/>
-      <c r="J71" t="inlineStr"/>
       <c r="K71" t="n">
         <v>0</v>
       </c>
@@ -4319,8 +4305,6 @@
           <t>thomas.maher@coates.com.au; cody.mitchell@coates.com.au; benjamin.vandenbroek@cemaust.com.au; david.moore@cemaust.com.au; John.Pickels@cemaust.com.au</t>
         </is>
       </c>
-      <c r="I72" t="inlineStr"/>
-      <c r="J72" t="inlineStr"/>
       <c r="K72" t="n">
         <v>0</v>
       </c>
@@ -4372,8 +4356,6 @@
           <t>thomas.maher@coates.com.au; cody.mitchell@coates.com.au; benjamin.vandenbroek@cemaust.com.au; david.moore@cemaust.com.au; John.Pickels@cemaust.com.au</t>
         </is>
       </c>
-      <c r="I73" t="inlineStr"/>
-      <c r="J73" t="inlineStr"/>
       <c r="K73" t="n">
         <v>0</v>
       </c>
@@ -4425,8 +4407,6 @@
           <t>thomas.maher@coates.com.au; cody.mitchell@coates.com.au; benjamin.vandenbroek@cemaust.com.au; david.moore@cemaust.com.au; John.Pickels@cemaust.com.au</t>
         </is>
       </c>
-      <c r="I74" t="inlineStr"/>
-      <c r="J74" t="inlineStr"/>
       <c r="K74" t="n">
         <v>0</v>
       </c>
@@ -4478,8 +4458,6 @@
           <t>thomas.maher@coates.com.au; cody.mitchell@coates.com.au; benjamin.vandenbroek@cemaust.com.au; david.moore@cemaust.com.au; John.Pickels@cemaust.com.au</t>
         </is>
       </c>
-      <c r="I75" t="inlineStr"/>
-      <c r="J75" t="inlineStr"/>
       <c r="K75" t="n">
         <v>0</v>
       </c>
@@ -4531,8 +4509,6 @@
           <t>grant.holdsworth@cemaust.com.au; hazel.barba@cemaust.com.au; carmen.groat@cemaust.com.au; daniel.osborne@cemaust.com.au; aaron.watts@cemaust.com.au; thomas.maher@coates.com.au; cody.mitchell@coates.com.au; adam.mcinnes@cemaust.com.au; kris.tierney@cemaust.com.au; melissa.cooper@cemaust.com.au; nicole.ward@cemaust.com.au</t>
         </is>
       </c>
-      <c r="I76" t="inlineStr"/>
-      <c r="J76" t="inlineStr"/>
       <c r="K76" t="n">
         <v>0</v>
       </c>
@@ -4584,8 +4560,6 @@
           <t>thomas.maher@coates.com.au; cody.mitchell@coates.com.au; benjamin.vandenbroek@cemaust.com.au; david.moore@cemaust.com.au; John.Pickels@cemaust.com.au</t>
         </is>
       </c>
-      <c r="I77" t="inlineStr"/>
-      <c r="J77" t="inlineStr"/>
       <c r="K77" t="n">
         <v>0</v>
       </c>
@@ -4637,8 +4611,6 @@
           <t>thomas.maher@coates.com.au; cody.mitchell@coates.com.au; benjamin.vandenbroek@cemaust.com.au; david.moore@cemaust.com.au; John.Pickels@cemaust.com.au</t>
         </is>
       </c>
-      <c r="I78" t="inlineStr"/>
-      <c r="J78" t="inlineStr"/>
       <c r="K78" t="n">
         <v>0</v>
       </c>
@@ -4690,8 +4662,6 @@
           <t>thomas.maher@coates.com.au; cody.mitchell@coates.com.au; benjamin.vandenbroek@cemaust.com.au; david.moore@cemaust.com.au; John.Pickels@cemaust.com.au</t>
         </is>
       </c>
-      <c r="I79" t="inlineStr"/>
-      <c r="J79" t="inlineStr"/>
       <c r="K79" t="n">
         <v>0</v>
       </c>
@@ -4733,14 +4703,11 @@
       <c r="F80" t="n">
         <v>14</v>
       </c>
-      <c r="G80" t="inlineStr"/>
       <c r="H80" t="inlineStr">
         <is>
           <t>thomas.maher@coates.com.au; cody.mitchell@coates.com.au; benjamin.vandenbroek@cemaust.com.au; david.moore@cemaust.com.au; John.Pickels@cemaust.com.au</t>
         </is>
       </c>
-      <c r="I80" t="inlineStr"/>
-      <c r="J80" t="inlineStr"/>
       <c r="K80" t="n">
         <v>0</v>
       </c>
@@ -4792,8 +4759,6 @@
           <t>thomas.maher@coates.com.au; cody.mitchell@coates.com.au; benjamin.vandenbroek@cemaust.com.au; david.moore@cemaust.com.au; John.Pickels@cemaust.com.au</t>
         </is>
       </c>
-      <c r="I81" t="inlineStr"/>
-      <c r="J81" t="inlineStr"/>
       <c r="K81" t="n">
         <v>0</v>
       </c>
@@ -4845,8 +4810,6 @@
           <t>thomas.maher@coates.com.au; cody.mitchell@coates.com.au; benjamin.vandenbroek@cemaust.com.au; david.moore@cemaust.com.au; John.Pickels@cemaust.com.au</t>
         </is>
       </c>
-      <c r="I82" t="inlineStr"/>
-      <c r="J82" t="inlineStr"/>
       <c r="K82" t="n">
         <v>0</v>
       </c>
@@ -4860,6 +4823,971 @@
           <t>Report in the body is today's, and still the current one (nothing generated) | Report ready for the email body (nothing generated) | Their own report is the only attachment (nothing attached) | No other company's information in the pack (found: (there is no report to read))</t>
         </is>
       </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>Cleanaway</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>External contractor</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>Not Generated</t>
+        </is>
+      </c>
+      <c r="E83" t="n">
+        <v>9</v>
+      </c>
+      <c r="F83" t="n">
+        <v>14</v>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>jayden.andrew@cleanaway.com.au</t>
+        </is>
+      </c>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>thomas.maher@coates.com.au; cody.mitchell@coates.com.au; benjamin.vandenbroek@cemaust.com.au; david.moore@cemaust.com.au; John.Pickels@cemaust.com.au</t>
+        </is>
+      </c>
+      <c r="I83" t="inlineStr"/>
+      <c r="J83" t="inlineStr"/>
+      <c r="K83" t="n">
+        <v>0</v>
+      </c>
+      <c r="L83" t="inlineStr">
+        <is>
+          <t>2026-08-05 12:25</t>
+        </is>
+      </c>
+      <c r="M83" t="inlineStr">
+        <is>
+          <t>Cleanaway holds nothing on hire today - no report to send. The folder and this record are made so the day is complete.</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>DGH Engineering</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>External contractor</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>Draft Ready</t>
+        </is>
+      </c>
+      <c r="E84" t="n">
+        <v>14</v>
+      </c>
+      <c r="F84" t="n">
+        <v>14</v>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>ross.gould@dgh.com.au; jadams@dgh.com.au; aburgun@dgh.com.au; btooma@dgh.com.au</t>
+        </is>
+      </c>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>thomas.maher@coates.com.au; cody.mitchell@coates.com.au; benjamin.vandenbroek@cemaust.com.au; david.moore@cemaust.com.au; John.Pickels@cemaust.com.au</t>
+        </is>
+      </c>
+      <c r="I84" t="inlineStr">
+        <is>
+          <t>DGH Engineering - On-Hire Report - 2026-08-05.html</t>
+        </is>
+      </c>
+      <c r="J84" t="inlineStr">
+        <is>
+          <t>DGH Engineering - On-Hire Report - 2026-08-05.pdf</t>
+        </is>
+      </c>
+      <c r="K84" t="n">
+        <v>5.16</v>
+      </c>
+      <c r="L84" t="inlineStr">
+        <is>
+          <t>2026-08-05 12:25</t>
+        </is>
+      </c>
+      <c r="M84" t="inlineStr"/>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>DKE Group</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>External contractor</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>Draft Ready</t>
+        </is>
+      </c>
+      <c r="E85" t="n">
+        <v>14</v>
+      </c>
+      <c r="F85" t="n">
+        <v>14</v>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>louis.miller@dkegroup.com.au; illy.reitsma@dkegroup.com.au; warren.wilson@dkegroup.com.au; tim.lalor@dkegroup.com.au</t>
+        </is>
+      </c>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>thomas.maher@coates.com.au; cody.mitchell@coates.com.au; benjamin.vandenbroek@cemaust.com.au; david.moore@cemaust.com.au; John.Pickels@cemaust.com.au</t>
+        </is>
+      </c>
+      <c r="I85" t="inlineStr">
+        <is>
+          <t>DKE Group - On-Hire Report - 2026-08-05.html</t>
+        </is>
+      </c>
+      <c r="J85" t="inlineStr">
+        <is>
+          <t>DKE Group - On-Hire Report - 2026-08-05.pdf</t>
+        </is>
+      </c>
+      <c r="K85" t="n">
+        <v>1.41</v>
+      </c>
+      <c r="L85" t="inlineStr">
+        <is>
+          <t>2026-08-05 12:25</t>
+        </is>
+      </c>
+      <c r="M85" t="inlineStr"/>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>High Risk Solutions</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>External contractor</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>Draft Ready</t>
+        </is>
+      </c>
+      <c r="E86" t="n">
+        <v>14</v>
+      </c>
+      <c r="F86" t="n">
+        <v>14</v>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>ca@highrisksolutions.com.au; david.nunn@highrisksolutions.com.au; jzuniga@highrisksolutions.com.au</t>
+        </is>
+      </c>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t>thomas.maher@coates.com.au; cody.mitchell@coates.com.au; benjamin.vandenbroek@cemaust.com.au; david.moore@cemaust.com.au; John.Pickels@cemaust.com.au</t>
+        </is>
+      </c>
+      <c r="I86" t="inlineStr">
+        <is>
+          <t>High Risk Solutions - On-Hire Report - 2026-08-05.html</t>
+        </is>
+      </c>
+      <c r="J86" t="inlineStr">
+        <is>
+          <t>High Risk Solutions - On-Hire Report - 2026-08-05.pdf</t>
+        </is>
+      </c>
+      <c r="K86" t="n">
+        <v>3.21</v>
+      </c>
+      <c r="L86" t="inlineStr">
+        <is>
+          <t>2026-08-05 12:25</t>
+        </is>
+      </c>
+      <c r="M86" t="inlineStr"/>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>Industec</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>External contractor</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>Draft Ready</t>
+        </is>
+      </c>
+      <c r="E87" t="n">
+        <v>14</v>
+      </c>
+      <c r="F87" t="n">
+        <v>14</v>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>m.clayton@industec.com.au</t>
+        </is>
+      </c>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>thomas.maher@coates.com.au; cody.mitchell@coates.com.au; benjamin.vandenbroek@cemaust.com.au; david.moore@cemaust.com.au; John.Pickels@cemaust.com.au</t>
+        </is>
+      </c>
+      <c r="I87" t="inlineStr">
+        <is>
+          <t>Industec - On-Hire Report - 2026-08-05.html</t>
+        </is>
+      </c>
+      <c r="J87" t="inlineStr">
+        <is>
+          <t>Industec - On-Hire Report - 2026-08-05.pdf</t>
+        </is>
+      </c>
+      <c r="K87" t="n">
+        <v>0.59</v>
+      </c>
+      <c r="L87" t="inlineStr">
+        <is>
+          <t>2026-08-05 12:25</t>
+        </is>
+      </c>
+      <c r="M87" t="inlineStr"/>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>Programmed</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>External contractor</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>Draft Ready</t>
+        </is>
+      </c>
+      <c r="E88" t="n">
+        <v>14</v>
+      </c>
+      <c r="F88" t="n">
+        <v>14</v>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>debra.rogers@programmed.com.au</t>
+        </is>
+      </c>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>thomas.maher@coates.com.au; cody.mitchell@coates.com.au; benjamin.vandenbroek@cemaust.com.au; david.moore@cemaust.com.au; John.Pickels@cemaust.com.au</t>
+        </is>
+      </c>
+      <c r="I88" t="inlineStr">
+        <is>
+          <t>Programmed - On-Hire Report - 2026-08-05.html</t>
+        </is>
+      </c>
+      <c r="J88" t="inlineStr">
+        <is>
+          <t>Programmed - On-Hire Report - 2026-08-05.pdf</t>
+        </is>
+      </c>
+      <c r="K88" t="n">
+        <v>5.23</v>
+      </c>
+      <c r="L88" t="inlineStr">
+        <is>
+          <t>2026-08-05 12:25</t>
+        </is>
+      </c>
+      <c r="M88" t="inlineStr"/>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>Synclift</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>External contractor</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>Draft Ready</t>
+        </is>
+      </c>
+      <c r="E89" t="n">
+        <v>14</v>
+      </c>
+      <c r="F89" t="n">
+        <v>14</v>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>jbeard@synclift.com.au; blynch@synclift.com.au</t>
+        </is>
+      </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>thomas.maher@coates.com.au; cody.mitchell@coates.com.au; benjamin.vandenbroek@cemaust.com.au; david.moore@cemaust.com.au; John.Pickels@cemaust.com.au</t>
+        </is>
+      </c>
+      <c r="I89" t="inlineStr">
+        <is>
+          <t>Synclift - On-Hire Report - 2026-08-05.html</t>
+        </is>
+      </c>
+      <c r="J89" t="inlineStr">
+        <is>
+          <t>Synclift - On-Hire Report - 2026-08-05.pdf</t>
+        </is>
+      </c>
+      <c r="K89" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="L89" t="inlineStr">
+        <is>
+          <t>2026-08-05 12:25</t>
+        </is>
+      </c>
+      <c r="M89" t="inlineStr"/>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>Tasman Rope Access</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>External contractor</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>Draft Ready</t>
+        </is>
+      </c>
+      <c r="E90" t="n">
+        <v>14</v>
+      </c>
+      <c r="F90" t="n">
+        <v>14</v>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>c.sheppardkadel@tasmanropeaccess.com</t>
+        </is>
+      </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>thomas.maher@coates.com.au; cody.mitchell@coates.com.au; benjamin.vandenbroek@cemaust.com.au; david.moore@cemaust.com.au; John.Pickels@cemaust.com.au</t>
+        </is>
+      </c>
+      <c r="I90" t="inlineStr">
+        <is>
+          <t>Tasman Rope Access - On-Hire Report - 2026-08-05.html</t>
+        </is>
+      </c>
+      <c r="J90" t="inlineStr">
+        <is>
+          <t>Tasman Rope Access - On-Hire Report - 2026-08-05.pdf</t>
+        </is>
+      </c>
+      <c r="K90" t="n">
+        <v>1.06</v>
+      </c>
+      <c r="L90" t="inlineStr">
+        <is>
+          <t>2026-08-05 12:25</t>
+        </is>
+      </c>
+      <c r="M90" t="inlineStr"/>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>Universal Cranes</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>External contractor</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>Draft Ready</t>
+        </is>
+      </c>
+      <c r="E91" t="n">
+        <v>14</v>
+      </c>
+      <c r="F91" t="n">
+        <v>14</v>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>joshua.breslin@universalcranes.com</t>
+        </is>
+      </c>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t>thomas.maher@coates.com.au; cody.mitchell@coates.com.au; benjamin.vandenbroek@cemaust.com.au; david.moore@cemaust.com.au; John.Pickels@cemaust.com.au</t>
+        </is>
+      </c>
+      <c r="I91" t="inlineStr">
+        <is>
+          <t>Universal Cranes - On-Hire Report - 2026-08-05.html</t>
+        </is>
+      </c>
+      <c r="J91" t="inlineStr">
+        <is>
+          <t>Universal Cranes - On-Hire Report - 2026-08-05.pdf</t>
+        </is>
+      </c>
+      <c r="K91" t="n">
+        <v>1.12</v>
+      </c>
+      <c r="L91" t="inlineStr">
+        <is>
+          <t>2026-08-05 12:25</t>
+        </is>
+      </c>
+      <c r="M91" t="inlineStr"/>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>Veolia Refractory</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>External contractor</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>Draft Ready</t>
+        </is>
+      </c>
+      <c r="E92" t="n">
+        <v>14</v>
+      </c>
+      <c r="F92" t="n">
+        <v>14</v>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>melissa.rowlands1@veolia.com; andrew.macloughlin@veolia.com; tim.lang1@veolia.com</t>
+        </is>
+      </c>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>thomas.maher@coates.com.au; cody.mitchell@coates.com.au; benjamin.vandenbroek@cemaust.com.au; david.moore@cemaust.com.au; John.Pickels@cemaust.com.au</t>
+        </is>
+      </c>
+      <c r="I92" t="inlineStr">
+        <is>
+          <t>Veolia Refractory - On-Hire Report - 2026-08-05.html</t>
+        </is>
+      </c>
+      <c r="J92" t="inlineStr">
+        <is>
+          <t>Veolia Refractory - On-Hire Report - 2026-08-05.pdf</t>
+        </is>
+      </c>
+      <c r="K92" t="n">
+        <v>5.16</v>
+      </c>
+      <c r="L92" t="inlineStr">
+        <is>
+          <t>2026-08-05 12:25</t>
+        </is>
+      </c>
+      <c r="M92" t="inlineStr"/>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>Xtreme Engineering</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>External contractor</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>Draft Ready</t>
+        </is>
+      </c>
+      <c r="E93" t="n">
+        <v>14</v>
+      </c>
+      <c r="F93" t="n">
+        <v>14</v>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>kkay@xtremeengineering.com.au; scotth@xtremeengineering.com.au</t>
+        </is>
+      </c>
+      <c r="H93" t="inlineStr">
+        <is>
+          <t>thomas.maher@coates.com.au; cody.mitchell@coates.com.au; benjamin.vandenbroek@cemaust.com.au; david.moore@cemaust.com.au; John.Pickels@cemaust.com.au</t>
+        </is>
+      </c>
+      <c r="I93" t="inlineStr">
+        <is>
+          <t>Xtreme Engineering - On-Hire Report - 2026-08-05.html</t>
+        </is>
+      </c>
+      <c r="J93" t="inlineStr">
+        <is>
+          <t>Xtreme Engineering - On-Hire Report - 2026-08-05.pdf</t>
+        </is>
+      </c>
+      <c r="K93" t="n">
+        <v>1.34</v>
+      </c>
+      <c r="L93" t="inlineStr">
+        <is>
+          <t>2026-08-05 12:25</t>
+        </is>
+      </c>
+      <c r="M93" t="inlineStr"/>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>Cement Australia</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>Client master report</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>Failed - Review Required</t>
+        </is>
+      </c>
+      <c r="E94" t="n">
+        <v>11</v>
+      </c>
+      <c r="F94" t="n">
+        <v>14</v>
+      </c>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>david.moore@cemaust.com.au; benjamin.vandenbroek@cemaust.com.au; john.pickels@cemaust.com.au</t>
+        </is>
+      </c>
+      <c r="H94" t="inlineStr">
+        <is>
+          <t>grant.holdsworth@cemaust.com.au; hazel.barba@cemaust.com.au; carmen.groat@cemaust.com.au; daniel.osborne@cemaust.com.au; aaron.watts@cemaust.com.au; thomas.maher@coates.com.au; cody.mitchell@coates.com.au; adam.mcinnes@cemaust.com.au; kris.tierney@cemaust.com.au; melissa.cooper@cemaust.com.au; nicole.ward@cemaust.com.au</t>
+        </is>
+      </c>
+      <c r="I94" t="inlineStr"/>
+      <c r="J94" t="inlineStr">
+        <is>
+          <t>Cement Australia On-Hire Report - 2026-08-05.pdf</t>
+        </is>
+      </c>
+      <c r="K94" t="n">
+        <v>0</v>
+      </c>
+      <c r="L94" t="inlineStr">
+        <is>
+          <t>2026-08-05 12:25</t>
+        </is>
+      </c>
+      <c r="M94" t="inlineStr">
+        <is>
+          <t>Daily Safety &amp; Compliance Report has no PDF - it was not built for 05 Aug 2026 | Daily Cost Tracking Report has no PDF - it was not built for 05 Aug 2026 | Site Plant Report has no PDF - it was not built for 05 Aug 2026 | Consumables Usage Report has no PDF - it was not built for 05 Aug 2026 | Report in the body is today's, and still the current one (nothing generated) | Report ready for the email body (nothing generated) | All five Cement attachments present (missing: Daily Safety &amp; Compliance Report, Daily Cost Tracking Report, Site Plant Report, Consumables Usage Report)</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>Bosch Rexroth</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>External contractor</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>Draft Ready</t>
+        </is>
+      </c>
+      <c r="E95" t="n">
+        <v>14</v>
+      </c>
+      <c r="F95" t="n">
+        <v>14</v>
+      </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>gerhardus.vanderwesthuizen@boschrexroth.com.au</t>
+        </is>
+      </c>
+      <c r="H95" t="inlineStr">
+        <is>
+          <t>thomas.maher@coates.com.au; cody.mitchell@coates.com.au; benjamin.vandenbroek@cemaust.com.au; david.moore@cemaust.com.au; John.Pickels@cemaust.com.au</t>
+        </is>
+      </c>
+      <c r="I95" t="inlineStr">
+        <is>
+          <t>Bosch Rexroth - On-Hire Report - 2026-08-05.html</t>
+        </is>
+      </c>
+      <c r="J95" t="inlineStr">
+        <is>
+          <t>Bosch Rexroth - On-Hire Report - 2026-08-05.pdf</t>
+        </is>
+      </c>
+      <c r="K95" t="n">
+        <v>0.64</v>
+      </c>
+      <c r="L95" t="inlineStr">
+        <is>
+          <t>2026-08-05 12:25</t>
+        </is>
+      </c>
+      <c r="M95" t="inlineStr"/>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>Industrial Rescue</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>External contractor</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>Draft Ready</t>
+        </is>
+      </c>
+      <c r="E96" t="n">
+        <v>14</v>
+      </c>
+      <c r="F96" t="n">
+        <v>14</v>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>chris.short@iretcq.com</t>
+        </is>
+      </c>
+      <c r="H96" t="inlineStr">
+        <is>
+          <t>thomas.maher@coates.com.au; cody.mitchell@coates.com.au; benjamin.vandenbroek@cemaust.com.au; david.moore@cemaust.com.au; John.Pickels@cemaust.com.au</t>
+        </is>
+      </c>
+      <c r="I96" t="inlineStr">
+        <is>
+          <t>Industrial Rescue - On-Hire Report - 2026-08-05.html</t>
+        </is>
+      </c>
+      <c r="J96" t="inlineStr">
+        <is>
+          <t>Industrial Rescue - On-Hire Report - 2026-08-05.pdf</t>
+        </is>
+      </c>
+      <c r="K96" t="n">
+        <v>0.89</v>
+      </c>
+      <c r="L96" t="inlineStr">
+        <is>
+          <t>2026-08-05 12:25</t>
+        </is>
+      </c>
+      <c r="M96" t="inlineStr"/>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>Filtercare</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>External contractor</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>Draft Ready</t>
+        </is>
+      </c>
+      <c r="E97" t="n">
+        <v>14</v>
+      </c>
+      <c r="F97" t="n">
+        <v>14</v>
+      </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>admin@industec.com.au</t>
+        </is>
+      </c>
+      <c r="H97" t="inlineStr">
+        <is>
+          <t>thomas.maher@coates.com.au; cody.mitchell@coates.com.au; benjamin.vandenbroek@cemaust.com.au; david.moore@cemaust.com.au; John.Pickels@cemaust.com.au</t>
+        </is>
+      </c>
+      <c r="I97" t="inlineStr">
+        <is>
+          <t>Filtercare - On-Hire Report - 2026-08-05.html</t>
+        </is>
+      </c>
+      <c r="J97" t="inlineStr">
+        <is>
+          <t>Filtercare - On-Hire Report - 2026-08-05.pdf</t>
+        </is>
+      </c>
+      <c r="K97" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="L97" t="inlineStr">
+        <is>
+          <t>2026-08-05 12:25</t>
+        </is>
+      </c>
+      <c r="M97" t="inlineStr"/>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>Aestec</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>External contractor</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>Draft Ready</t>
+        </is>
+      </c>
+      <c r="E98" t="n">
+        <v>14</v>
+      </c>
+      <c r="F98" t="n">
+        <v>14</v>
+      </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>accounts@aestec.com.au</t>
+        </is>
+      </c>
+      <c r="H98" t="inlineStr">
+        <is>
+          <t>thomas.maher@coates.com.au; cody.mitchell@coates.com.au; benjamin.vandenbroek@cemaust.com.au; david.moore@cemaust.com.au; John.Pickels@cemaust.com.au</t>
+        </is>
+      </c>
+      <c r="I98" t="inlineStr">
+        <is>
+          <t>Aestec - On-Hire Report - 2026-08-05.html</t>
+        </is>
+      </c>
+      <c r="J98" t="inlineStr">
+        <is>
+          <t>Aestec - On-Hire Report - 2026-08-05.pdf</t>
+        </is>
+      </c>
+      <c r="K98" t="n">
+        <v>0.48</v>
+      </c>
+      <c r="L98" t="inlineStr">
+        <is>
+          <t>2026-08-05 12:25</t>
+        </is>
+      </c>
+      <c r="M98" t="inlineStr"/>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>Cutrite</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>External contractor</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>Draft Ready</t>
+        </is>
+      </c>
+      <c r="E99" t="n">
+        <v>14</v>
+      </c>
+      <c r="F99" t="n">
+        <v>14</v>
+      </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>matt@cutrite.net.au</t>
+        </is>
+      </c>
+      <c r="H99" t="inlineStr">
+        <is>
+          <t>thomas.maher@coates.com.au; cody.mitchell@coates.com.au; benjamin.vandenbroek@cemaust.com.au; david.moore@cemaust.com.au; John.Pickels@cemaust.com.au</t>
+        </is>
+      </c>
+      <c r="I99" t="inlineStr">
+        <is>
+          <t>Cutrite - On-Hire Report - 2026-08-05.html</t>
+        </is>
+      </c>
+      <c r="J99" t="inlineStr">
+        <is>
+          <t>Cutrite - On-Hire Report - 2026-08-05.pdf</t>
+        </is>
+      </c>
+      <c r="K99" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="L99" t="inlineStr">
+        <is>
+          <t>2026-08-05 12:25</t>
+        </is>
+      </c>
+      <c r="M99" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>